<commit_message>
fix: remove legacy field from Excel template guide
</commit_message>
<xml_diff>
--- a/public/templates/menu-import/menu-template.xlsx
+++ b/public/templates/menu-import/menu-template.xlsx
@@ -92,10 +92,10 @@
     <t>isAvailable accepte true ou false. Si la cellule est vide, la valeur true est utilisée.</t>
   </si>
   <si>
-    <t>Préparation</t>
-  </si>
-  <si>
-    <t>Ne renseignez pas preparationTime : cette colonne ne fait pas partie de l’import.</t>
+    <t>Temps de préparation</t>
+  </si>
+  <si>
+    <t>Cette information n’est pas demandée dans ce modèle.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
feat: ajouter la prise en charge des catégories de menu dynamiques et améliorer le traitement des fichiers CSV
</commit_message>
<xml_diff>
--- a/public/templates/menu-import/menu-template.xlsx
+++ b/public/templates/menu-import/menu-template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="29">
   <si>
     <t>externalId</t>
   </si>
@@ -62,40 +62,43 @@
     <t>Desserts</t>
   </si>
   <si>
-    <t>Règle</t>
-  </si>
-  <si>
-    <t>Explication</t>
-  </si>
-  <si>
-    <t>Colonnes obligatoires</t>
-  </si>
-  <si>
-    <t>externalId, name et price doivent être renseignées pour chaque plat.</t>
-  </si>
-  <si>
-    <t>Colonnes optionnelles</t>
-  </si>
-  <si>
-    <t>description, category, isAvailable et image peuvent être laissées vides.</t>
-  </si>
-  <si>
-    <t>Images Excel</t>
-  </si>
-  <si>
-    <t>Insérez une image dans la cellule de la colonne image sur la ligne du plat correspondant.</t>
-  </si>
-  <si>
-    <t>Disponibilité</t>
-  </si>
-  <si>
-    <t>isAvailable accepte true ou false. Si la cellule est vide, la valeur true est utilisée.</t>
-  </si>
-  <si>
-    <t>Temps de préparation</t>
-  </si>
-  <si>
-    <t>Cette information n’est pas demandée dans ce modèle.</t>
+    <t>Champ</t>
+  </si>
+  <si>
+    <t>Statut</t>
+  </si>
+  <si>
+    <t>Note courte</t>
+  </si>
+  <si>
+    <t>Obligatoire</t>
+  </si>
+  <si>
+    <t>Identifiant unique du plat.</t>
+  </si>
+  <si>
+    <t>Nom affiché du plat.</t>
+  </si>
+  <si>
+    <t>Prix positif, ex. 12.50.</t>
+  </si>
+  <si>
+    <t>description, category</t>
+  </si>
+  <si>
+    <t>Optionnels</t>
+  </si>
+  <si>
+    <t>Peuvent rester vides.</t>
+  </si>
+  <si>
+    <t>Optionnel</t>
+  </si>
+  <si>
+    <t>true ou false ; vide = disponible.</t>
+  </si>
+  <si>
+    <t>Insérez l’image sur la ligne du plat.</t>
   </si>
 </sst>
 </file>
@@ -625,59 +628,89 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="90" customWidth="1"/>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C1" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="3" t="s">
+    </row>
+    <row r="5" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="B5" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>